<commit_message>
#28 Client BOM 10 Boards Quantity Updated
</commit_message>
<xml_diff>
--- a/Design Files/OLED-v2.0/BOM/Client_BOM_OLED-v2.0.xlsx
+++ b/Design Files/OLED-v2.0/BOM/Client_BOM_OLED-v2.0.xlsx
@@ -12,14 +12,14 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="10 Boards" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="108">
   <si>
     <t>Component list</t>
   </si>
@@ -312,36 +312,12 @@
     <t>Value</t>
   </si>
   <si>
-    <t>Quantity (5 Boards)</t>
-  </si>
-  <si>
-    <t>Links</t>
-  </si>
-  <si>
-    <t>Unit Cost (5 Boards)</t>
-  </si>
-  <si>
-    <t>Total Cost (5 Boards)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Component Cost </t>
-  </si>
-  <si>
-    <t>Single Board Cost</t>
-  </si>
-  <si>
     <t>Remarks</t>
   </si>
   <si>
-    <t>Digikey</t>
-  </si>
-  <si>
     <t>CL05A475KP5NRNC</t>
   </si>
   <si>
-    <t>Custom Supplier</t>
-  </si>
-  <si>
     <t>Peripheral</t>
   </si>
   <si>
@@ -364,18 +340,19 @@
   </si>
   <si>
     <t>XFCN</t>
+  </si>
+  <si>
+    <t>Quantity (10 Boards)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="3">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
-    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -515,14 +492,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="14"/>
       <name val="Calibri"/>
@@ -556,7 +525,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -764,40 +733,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -951,22 +891,14 @@
     <xf numFmtId="0" fontId="19" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="3" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="20" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="20" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -978,23 +910,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1020,13 +937,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>15</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>47625</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>19942</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>1905000</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>171450</xdr:rowOff>
@@ -1334,7 +1251,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -1348,13 +1265,10 @@
     <col min="10" max="10" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.140625" customWidth="1"/>
-    <col min="14" max="14" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="29.42578125" customWidth="1"/>
+    <col min="13" max="13" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1364,15 +1278,12 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="64"/>
-      <c r="O1" s="64"/>
-      <c r="P1" s="64"/>
-    </row>
-    <row r="2" spans="1:16" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
+    </row>
+    <row r="2" spans="1:13" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="20"/>
       <c r="C2" s="41"/>
@@ -1389,12 +1300,9 @@
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="38"/>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M2" s="38"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="21"/>
       <c r="C3" s="42"/>
@@ -1411,12 +1319,9 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="65"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M3" s="62"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="21"/>
       <c r="C4" s="42"/>
@@ -1433,12 +1338,9 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
-      <c r="P4" s="66"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M4" s="63"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="21"/>
       <c r="C5" s="42"/>
@@ -1455,12 +1357,9 @@
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-      <c r="P5" s="66"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M5" s="63"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="22"/>
       <c r="C6" s="43"/>
@@ -1473,12 +1372,9 @@
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
-      <c r="P6" s="66"/>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M6" s="63"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="23"/>
       <c r="C7" s="44"/>
@@ -1491,12 +1387,9 @@
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
-      <c r="N7" s="7"/>
-      <c r="O7" s="7"/>
-      <c r="P7" s="66"/>
-    </row>
-    <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M7" s="63"/>
+    </row>
+    <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="26"/>
       <c r="C8" s="45"/>
@@ -1509,12 +1402,9 @@
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="7"/>
-      <c r="P8" s="66"/>
-    </row>
-    <row r="9" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M8" s="63"/>
+    </row>
+    <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="29" t="s">
         <v>4</v>
@@ -1547,22 +1437,13 @@
         <v>89</v>
       </c>
       <c r="L9" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="M9" s="29" t="s">
         <v>97</v>
       </c>
-      <c r="M9" s="29" t="s">
-        <v>98</v>
-      </c>
-      <c r="N9" s="29" t="s">
-        <v>99</v>
-      </c>
-      <c r="O9" s="29" t="s">
-        <v>100</v>
-      </c>
-      <c r="P9" s="29" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="52">
         <f>ROW(B10) - ROW($B$9)</f>
@@ -1596,22 +1477,12 @@
         <v>4</v>
       </c>
       <c r="L10" s="36">
-        <f>K10*5</f>
-        <v>20</v>
-      </c>
-      <c r="M10" s="62" t="s">
-        <v>104</v>
-      </c>
-      <c r="N10" s="58">
-        <v>7.3999999999999996E-2</v>
-      </c>
-      <c r="O10" s="58">
-        <f>N10*L10</f>
-        <v>1.48</v>
-      </c>
-      <c r="P10" s="36"/>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+        <f>K10*10</f>
+        <v>40</v>
+      </c>
+      <c r="M10" s="36"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="54">
         <f t="shared" ref="B11:B26" si="0">ROW(B11) - ROW($B$9)</f>
@@ -1644,23 +1515,13 @@
       <c r="K11" s="37">
         <v>4</v>
       </c>
-      <c r="L11" s="37">
-        <f t="shared" ref="L11" si="1">K11*5</f>
-        <v>20</v>
-      </c>
-      <c r="M11" s="62" t="s">
-        <v>104</v>
-      </c>
-      <c r="N11" s="59">
-        <v>7.9000000000000001E-2</v>
-      </c>
-      <c r="O11" s="59">
-        <f t="shared" ref="O11" si="2">N11*L11</f>
-        <v>1.58</v>
-      </c>
-      <c r="P11" s="37"/>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="L11" s="36">
+        <f t="shared" ref="L11:L26" si="1">K11*10</f>
+        <v>40</v>
+      </c>
+      <c r="M11" s="37"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="52">
         <f>ROW(B12) - ROW($B$9)</f>
@@ -1682,7 +1543,7 @@
         <v>60</v>
       </c>
       <c r="H12" s="36" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="I12" s="36" t="s">
         <v>71</v>
@@ -1694,22 +1555,12 @@
         <v>1</v>
       </c>
       <c r="L12" s="36">
-        <f>K12*5</f>
-        <v>5</v>
-      </c>
-      <c r="M12" s="62" t="s">
-        <v>104</v>
-      </c>
-      <c r="N12" s="58">
-        <v>0.28000000000000003</v>
-      </c>
-      <c r="O12" s="58">
-        <f>N12*L12</f>
-        <v>1.4000000000000001</v>
-      </c>
-      <c r="P12" s="36"/>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="M12" s="36"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="54">
         <f t="shared" si="0"/>
@@ -1742,23 +1593,13 @@
       <c r="K13" s="37">
         <v>1</v>
       </c>
-      <c r="L13" s="37">
-        <f t="shared" ref="L13" si="3">K13*5</f>
-        <v>5</v>
-      </c>
-      <c r="M13" s="62" t="s">
-        <v>104</v>
-      </c>
-      <c r="N13" s="59">
-        <v>0.21</v>
-      </c>
-      <c r="O13" s="59">
-        <f t="shared" ref="O13" si="4">N13*L13</f>
-        <v>1.05</v>
-      </c>
-      <c r="P13" s="37"/>
-    </row>
-    <row r="14" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="L13" s="36">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="M13" s="37"/>
+    </row>
+    <row r="14" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="52">
         <f>ROW(B14) - ROW($B$9)</f>
@@ -1792,21 +1633,12 @@
         <v>1</v>
       </c>
       <c r="L14" s="36">
-        <f>K14*5</f>
-        <v>5</v>
-      </c>
-      <c r="M14" s="63" t="s">
-        <v>106</v>
-      </c>
-      <c r="N14" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="O14" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="P14" s="36"/>
-    </row>
-    <row r="15" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="M14" s="36"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="54">
         <f t="shared" si="0"/>
@@ -1839,47 +1671,38 @@
       <c r="K15" s="56">
         <v>1</v>
       </c>
-      <c r="L15" s="56">
-        <f t="shared" ref="L15" si="5">K15*5</f>
-        <v>5</v>
-      </c>
-      <c r="M15" s="63" t="s">
-        <v>106</v>
-      </c>
-      <c r="N15" s="56" t="s">
-        <v>95</v>
-      </c>
-      <c r="O15" s="56" t="s">
-        <v>95</v>
-      </c>
-      <c r="P15" s="37"/>
-    </row>
-    <row r="16" spans="1:16" ht="48" x14ac:dyDescent="0.25">
+      <c r="L15" s="36">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="M15" s="37"/>
+    </row>
+    <row r="16" spans="1:13" ht="48" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="52">
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
       <c r="C16" s="55" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="D16" s="36" t="s">
         <v>22</v>
       </c>
       <c r="E16" s="36" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="F16" s="36" t="s">
         <v>90</v>
       </c>
       <c r="G16" s="36" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="H16" s="36" t="s">
         <v>95</v>
       </c>
       <c r="I16" s="36" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="J16" s="36" t="s">
         <v>95</v>
@@ -1888,21 +1711,12 @@
         <v>1</v>
       </c>
       <c r="L16" s="36">
-        <f>K16*5</f>
-        <v>5</v>
-      </c>
-      <c r="M16" s="63" t="s">
-        <v>106</v>
-      </c>
-      <c r="N16" s="56" t="s">
-        <v>95</v>
-      </c>
-      <c r="O16" s="56" t="s">
-        <v>95</v>
-      </c>
-      <c r="P16" s="36"/>
-    </row>
-    <row r="17" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="M16" s="36"/>
+    </row>
+    <row r="17" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="54">
         <f t="shared" si="0"/>
@@ -1933,22 +1747,13 @@
       <c r="K17" s="37">
         <v>1</v>
       </c>
-      <c r="L17" s="37">
-        <f t="shared" ref="L17" si="6">K17*5</f>
-        <v>5</v>
-      </c>
-      <c r="M17" s="63" t="s">
-        <v>106</v>
-      </c>
-      <c r="N17" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="O17" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="P17" s="37"/>
-    </row>
-    <row r="18" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="L17" s="36">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="M17" s="37"/>
+    </row>
+    <row r="18" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="52">
         <f>ROW(B18) - ROW($B$9)</f>
@@ -1980,21 +1785,12 @@
         <v>1</v>
       </c>
       <c r="L18" s="36">
-        <f>K18*5</f>
-        <v>5</v>
-      </c>
-      <c r="M18" s="63" t="s">
-        <v>106</v>
-      </c>
-      <c r="N18" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="O18" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="P18" s="36"/>
-    </row>
-    <row r="19" spans="1:16" ht="36" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="M18" s="36"/>
+    </row>
+    <row r="19" spans="1:13" ht="36" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="54">
         <f t="shared" si="0"/>
@@ -2025,22 +1821,13 @@
       <c r="K19" s="37">
         <v>1</v>
       </c>
-      <c r="L19" s="37">
-        <f t="shared" ref="L19" si="7">K19*5</f>
-        <v>5</v>
-      </c>
-      <c r="M19" s="63" t="s">
-        <v>106</v>
-      </c>
-      <c r="N19" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="O19" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="P19" s="37"/>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="L19" s="36">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="M19" s="37"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="52">
         <f>ROW(B20) - ROW($B$9)</f>
@@ -2074,22 +1861,12 @@
         <v>4</v>
       </c>
       <c r="L20" s="36">
-        <f>K20*5</f>
-        <v>20</v>
-      </c>
-      <c r="M20" s="62" t="s">
-        <v>104</v>
-      </c>
-      <c r="N20" s="58">
-        <v>0.28799999999999998</v>
-      </c>
-      <c r="O20" s="58">
-        <f>N20*L20</f>
-        <v>5.76</v>
-      </c>
-      <c r="P20" s="36"/>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+      <c r="M20" s="36"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="54">
         <f t="shared" si="0"/>
@@ -2122,23 +1899,13 @@
       <c r="K21" s="37">
         <v>1</v>
       </c>
-      <c r="L21" s="37">
-        <f t="shared" ref="L21" si="8">K21*5</f>
-        <v>5</v>
-      </c>
-      <c r="M21" s="62" t="s">
-        <v>104</v>
-      </c>
-      <c r="N21" s="59">
-        <v>0.1</v>
-      </c>
-      <c r="O21" s="59">
-        <f t="shared" ref="O21" si="9">N21*L21</f>
-        <v>0.5</v>
-      </c>
-      <c r="P21" s="37"/>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="L21" s="36">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="M21" s="37"/>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="52">
         <f>ROW(B22) - ROW($B$9)</f>
@@ -2172,22 +1939,12 @@
         <v>1</v>
       </c>
       <c r="L22" s="36">
-        <f>K22*5</f>
-        <v>5</v>
-      </c>
-      <c r="M22" s="62" t="s">
-        <v>104</v>
-      </c>
-      <c r="N22" s="58">
-        <v>0.1</v>
-      </c>
-      <c r="O22" s="58">
-        <f>N22*L22</f>
-        <v>0.5</v>
-      </c>
-      <c r="P22" s="36"/>
-    </row>
-    <row r="23" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="M22" s="36"/>
+    </row>
+    <row r="23" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="54">
         <f t="shared" si="0"/>
@@ -2220,22 +1977,13 @@
       <c r="K23" s="37">
         <v>1</v>
       </c>
-      <c r="L23" s="37">
-        <f t="shared" ref="L23" si="10">K23*5</f>
-        <v>5</v>
-      </c>
-      <c r="M23" s="63" t="s">
-        <v>106</v>
-      </c>
-      <c r="N23" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="O23" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="P23" s="37"/>
-    </row>
-    <row r="24" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="L23" s="36">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="M23" s="37"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="52">
         <f>ROW(B24) - ROW($B$9)</f>
@@ -2268,22 +2016,13 @@
       <c r="K24" s="57">
         <v>1</v>
       </c>
-      <c r="L24" s="57">
-        <f>K24*5</f>
-        <v>5</v>
-      </c>
-      <c r="M24" s="63" t="s">
-        <v>106</v>
-      </c>
-      <c r="N24" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="O24" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="P24" s="36"/>
-    </row>
-    <row r="25" spans="1:16" ht="36" x14ac:dyDescent="0.25">
+      <c r="L24" s="36">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="M24" s="36"/>
+    </row>
+    <row r="25" spans="1:13" ht="36" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" s="54">
         <f t="shared" si="0"/>
@@ -2316,47 +2055,38 @@
       <c r="K25" s="37">
         <v>3</v>
       </c>
-      <c r="L25" s="37">
-        <f t="shared" ref="L25:L26" si="11">K25*5</f>
-        <v>15</v>
-      </c>
-      <c r="M25" s="63" t="s">
-        <v>106</v>
-      </c>
-      <c r="N25" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="O25" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="P25" s="37"/>
-    </row>
-    <row r="26" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L25" s="36">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+      <c r="M25" s="37"/>
+    </row>
+    <row r="26" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="54">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="C26" s="53" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="D26" s="37" t="s">
         <v>95</v>
       </c>
       <c r="E26" s="37" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="F26" s="36" t="s">
         <v>95</v>
       </c>
       <c r="G26" s="37" t="s">
-        <v>109</v>
-      </c>
-      <c r="H26" s="69" t="s">
+        <v>101</v>
+      </c>
+      <c r="H26" s="59" t="s">
         <v>95</v>
       </c>
       <c r="I26" s="37" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="J26" s="37" t="s">
         <v>95</v>
@@ -2364,22 +2094,13 @@
       <c r="K26" s="37">
         <v>1</v>
       </c>
-      <c r="L26" s="37">
-        <f t="shared" si="11"/>
-        <v>5</v>
-      </c>
-      <c r="M26" s="63" t="s">
-        <v>106</v>
-      </c>
-      <c r="N26" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="O26" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="P26" s="70"/>
-    </row>
-    <row r="27" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L26" s="36">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="M26" s="60"/>
+    </row>
+    <row r="27" spans="1:13" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="31"/>
       <c r="C27" s="46"/>
@@ -2391,18 +2112,10 @@
       <c r="I27" s="34"/>
       <c r="J27" s="35"/>
       <c r="K27" s="35"/>
-      <c r="L27" s="67" t="s">
-        <v>101</v>
-      </c>
-      <c r="M27" s="68"/>
-      <c r="N27" s="68"/>
-      <c r="O27" s="60">
-        <f>SUM(O10:O25)</f>
-        <v>12.27</v>
-      </c>
-      <c r="P27" s="39"/>
-    </row>
-    <row r="28" spans="1:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L27" s="58"/>
+      <c r="M27" s="39"/>
+    </row>
+    <row r="28" spans="1:13" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="24"/>
       <c r="C28" s="47"/>
@@ -2414,35 +2127,16 @@
       <c r="I28" s="9"/>
       <c r="J28" s="9"/>
       <c r="K28" s="9"/>
-      <c r="L28" s="67" t="s">
-        <v>102</v>
-      </c>
-      <c r="M28" s="68"/>
-      <c r="N28" s="68"/>
-      <c r="O28" s="61">
-        <f>O27/5</f>
-        <v>2.4539999999999997</v>
-      </c>
-      <c r="P28" s="40"/>
+      <c r="L28" s="58"/>
+      <c r="M28" s="40"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="J1:P1"/>
-    <mergeCell ref="P3:P8"/>
-    <mergeCell ref="L27:N27"/>
-    <mergeCell ref="L28:N28"/>
+  <mergeCells count="2">
+    <mergeCell ref="J1:M1"/>
+    <mergeCell ref="M3:M8"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="M10" r:id="rId1"/>
-    <hyperlink ref="M11" r:id="rId2"/>
-    <hyperlink ref="M12" r:id="rId3"/>
-    <hyperlink ref="M13" r:id="rId4"/>
-    <hyperlink ref="M20" r:id="rId5"/>
-    <hyperlink ref="M21" r:id="rId6"/>
-    <hyperlink ref="M22" r:id="rId7"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId8"/>
-  <drawing r:id="rId9"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>